<commit_message>
bug fixes and improvements
</commit_message>
<xml_diff>
--- a/outputs/allocations.xlsx
+++ b/outputs/allocations.xlsx
@@ -7,14 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="All results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="13 Oct (Tue) 6.00pm - 8.00pm @ " sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="17 Oct (Sat) 1.30pm - 3.15pm @ " sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="17 Oct (Sat) 3.15pm - 5.00pm @ " sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="18 Oct (Sun) 10.30am - 11.45am " sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="18 Oct (Sun) 11.45am - 1.00pm @" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="18 Oct (Sun) 9.00am - 10.30am @" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Not members" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="All allocated" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tue 13 Oct 6.00pm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sat 17 Oct 1.30pm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sat 17 Oct 3.15pm" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sun 18 Oct 10.30am" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sun 18 Oct 11.45am" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sun 18 Oct 9.00am (coached)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Rejected" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,23 +420,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>UCL email address</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>Allocated session</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Session (full)</t>
         </is>
       </c>
     </row>
@@ -448,10 +453,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zcesttu@ucl.ac.uk</t>
+          <t>Tinnakrit.tuaicharoen.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -460,15 +470,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tom Stevens</t>
+          <t>Thomas Stevens</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zcbttj7@ucl.ac.uk</t>
+          <t>thomas.stevens.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -477,15 +492,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vu Ngo</t>
+          <t>Ngo Hoai Vu</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>zczqgox@ucl.ac.uk</t>
+          <t>hoai.ngo.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -499,10 +519,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>uczcyha@ucl.ac.uk</t>
+          <t>Ying.han.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -516,10 +541,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>stnzinq@ucl.ac.uk</t>
+          <t>yan.lin.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -533,10 +563,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>zccanai@ucl.ac.uk</t>
+          <t>arjun.nair.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -545,15 +580,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wen-Han Chuang</t>
+          <t xml:space="preserve">WenHan Chuang </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>uceswc8@ucl.ac.uk</t>
+          <t>wen-han.chuang.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -562,15 +602,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wei Haozhan</t>
+          <t>haozhan Wei</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ucbv936@ucl.ac.uk</t>
+          <t>haozhan.wei.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -579,15 +624,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Huang Yalan</t>
+          <t>Yalan Huang</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>zczquav@ucl.ac.uk</t>
+          <t>yalan.huang.23@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -596,15 +646,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Garry Vignarajah</t>
+          <t xml:space="preserve">Garry Vignarajah </t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>zcemgvi@ucl.ac.uk</t>
+          <t>garry.vignarajah.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -613,15 +668,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gordon Zhang</t>
+          <t>Boyu Zhang</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>zcembz4@ucl.ac.uk</t>
+          <t>boyu.zhang.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -630,15 +690,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Zhang Botao</t>
+          <t>Botao Zhang</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>zcembz2@ucl.ac.uk</t>
+          <t>botao.zhang.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -647,15 +712,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wu, Szu-Min</t>
+          <t>SZU MIN WU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ucenwuj@ucl.ac.uk</t>
+          <t>szu-min.wu.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -669,10 +739,15 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ucabdp5@ucl.ac.uk</t>
+          <t>darren.prasetya.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -686,10 +761,15 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ucnwiul@ucl.ac.uk</t>
+          <t>chin-chia.liu.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -698,15 +778,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Skye Chang</t>
+          <t>Skye H. Y. Chang</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ucjvhc1@ucl.ac.uk</t>
+          <t>hung-yi.chang.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -715,15 +800,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Wang Sbrace</t>
+          <t>David Wang</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>stnzj39@ucl.ac.uk</t>
+          <t>david.wang.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -732,15 +822,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Li Teresa</t>
+          <t>Teresa Li</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>zczqj84@ucl.ac.uk</t>
+          <t>jingtong.li.23@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -749,15 +844,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Chou, Ying Xuan</t>
+          <t>Ying Xuan Chou</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>smgxyc0@ucl.ac.uk</t>
+          <t>ying.chou.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -771,10 +871,15 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>zcahitt@ucl.ac.uk</t>
+          <t>ambuj.mittal.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -783,15 +888,20 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Zhu Mono</t>
+          <t>Mono(Yuliang) Zhu</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>zczv022@ucl.ac.uk</t>
+          <t>yuliang.zhu.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -800,15 +910,20 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Lih Jun Wong</t>
+          <t xml:space="preserve">Lih Jun Wong </t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>rmjwjwo@ucl.ac.uk</t>
+          <t>lih.wong.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -817,15 +932,20 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tian Yihan</t>
+          <t>Yihan Tian</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>zcibyti@ucl.ac.uk</t>
+          <t>yihan.tian.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -834,15 +954,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sun Tianhao</t>
+          <t>Tianhao Sun</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>zchats7@ucl.ac.uk</t>
+          <t>tianhao.sun.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -856,10 +981,15 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>zcabvl0@ucl.ac.uk</t>
+          <t>vernados.lin.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -873,10 +1003,15 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>yjmsjg2@ucl.ac.uk</t>
+          <t>judyta.gorska.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -885,15 +1020,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Yieh, Cynthia</t>
+          <t>Cynthia Yieh</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>dtnzxcy@ucl.ac.uk</t>
+          <t>xin-yu.yieh.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -902,15 +1042,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Guo, Jia-Liang</t>
+          <t>Jialiang Guo</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ucabuog@ucl.ac.uk</t>
+          <t>jia-liang.guo.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -919,15 +1064,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hyunwoo Oh</t>
+          <t>HYUNWOO Oh</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>zcahhxx@ucl.ac.uk</t>
+          <t>Hyunwoo.oh.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -936,15 +1086,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ellie Tsang</t>
+          <t xml:space="preserve">Ellie Tsang </t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>stnzct2@ucl.ac.uk</t>
+          <t>ellie.tsang.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -958,10 +1113,15 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>uctysee@ucl.ac.uk</t>
+          <t>silas.eeles-nolle.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -975,10 +1135,15 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>zcabnhc@ucl.ac.uk</t>
+          <t>nok.chau.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -987,15 +1152,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Shi Camilla</t>
+          <t>Camilla Shi</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>zctpcs8@ucl.ac.uk</t>
+          <t>camilla.shi.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1004,15 +1174,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jin Yunxuan</t>
+          <t>Yunxuan Jin</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>zcfayji@ucl.ac.uk</t>
+          <t>yunxuan.jin.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -1021,15 +1196,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Chloe Mok</t>
+          <t>Mok Ho Yi Chloe</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>zctqhym@ucl.ac.uk</t>
+          <t>chloe.chloe.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1038,15 +1218,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Choi Stephanie</t>
+          <t>Lok Yee Choi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>xkgtych@ucl.ac.uk</t>
+          <t>stephanie.choi.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1055,15 +1240,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wang Bobby</t>
+          <t>Bobby Wang</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>stnzew2@ucl.ac.uk</t>
+          <t>enxun.wang.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1072,7 +1262,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Chen Celia</t>
+          <t>Zhihan Chen</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1081,6 +1271,11 @@
         </is>
       </c>
       <c r="C39" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1089,15 +1284,20 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Allen Sun</t>
+          <t>Weilun Sun</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>zcbewsu@ucl.ac.uk</t>
+          <t>allen.sun.24@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1111,10 +1311,15 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>zchaic3@ucl.ac.uk</t>
+          <t>ian.chau.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1123,15 +1328,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Shen Haocong</t>
+          <t>Haocong Shen</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>zcbt548@ucl.ac.uk</t>
+          <t>haocong.shen.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1145,10 +1355,15 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>zcemkc6@ucl.ac.uk</t>
+          <t>Keyi.Chen.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -1157,15 +1372,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Wen Serena</t>
+          <t>Zixun Wen</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>zceizw5@ucl.ac.uk</t>
+          <t>zixun.wen.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -1179,10 +1399,15 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>zccazba@ucl.ac.uk</t>
+          <t>betty.bao.23@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1191,15 +1416,20 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Angelina May</t>
+          <t xml:space="preserve">Angelina May </t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>zcemmay@ucl.ac.uk</t>
+          <t>angelina.may.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1213,10 +1443,15 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>wmhksqi@ucl.ac.uk</t>
+          <t>toto.qiao.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1230,10 +1465,15 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>zctlfag@ucl.ac.uk</t>
+          <t>macaela.agyare.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1247,10 +1487,15 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>zcbtafu@ucl.ac.uk</t>
+          <t>adriel.fung.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -1264,10 +1509,15 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>zcftnts@ucl.ac.uk</t>
+          <t>nicole.tsoi.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -1276,49 +1526,64 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Song Roger</t>
+          <t xml:space="preserve">Roger Song </t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>zceehs4@ucl.ac.uk</t>
+          <t>haoyu.song.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Zong Guanchu</t>
+          <t>Guanchu Zong</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>zcemgzo@ucl.ac.uk</t>
+          <t>guanchu.zong.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Lisa Cheok</t>
+          <t>Lisa Cheok Xin Yi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>zcablxy@ucl.ac.uk</t>
+          <t>lisa.cheok.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1337,6 +1602,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
       </c>
@@ -1344,7 +1614,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Wang Yiqi</t>
+          <t>Yiqi Wang</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1353,6 +1623,11 @@
         </is>
       </c>
       <c r="C55" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1361,15 +1636,20 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Yu Sidi</t>
+          <t>SIDI YU</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ucbv968@ucl.ac.uk</t>
+          <t>sidi.yu.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1383,10 +1663,15 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>zcftxgo@ucl.ac.uk</t>
+          <t>betty.gong.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1395,15 +1680,20 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Linda Cai</t>
+          <t>Liping Cai (Linda)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>qtnzlc4@ucl.ac.uk</t>
+          <t>liping.cai.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1412,15 +1702,20 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Sophia An</t>
+          <t>Yixuan An</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>zcibanb@ucl.ac.uk</t>
+          <t>sophia.an.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1434,10 +1729,15 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>zctp454@ucl.ac.uk</t>
+          <t>ryan.lee.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1451,12 +1751,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>zctqip0@ucl.ac.uk</t>
+          <t>ishaan.palsule.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
       </c>
     </row>
@@ -1468,29 +1773,39 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>zcecamp@ucl.ac.uk</t>
+          <t>kendrix.pineda.25@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Jeffrey Li</t>
+          <t>Chung Lai Li Jeffrey</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>zctqlip@ucl.ac.uk</t>
+          <t>jeffrey.li.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
       </c>
     </row>
@@ -1502,10 +1817,15 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>zcjthuj@ucl.ac.uk</t>
+          <t>Rayne.Zhu.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -1514,32 +1834,42 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Ge Xiaoxiao</t>
+          <t>Xiaoxiao Ge</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>uclqxge@ucl.ac.uk</t>
+          <t>xiaoxiao.ge.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>UNALLOCATED</t>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Sakai Yuki</t>
+          <t>Yuki Sakai</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>uclqysa@ucl.ac.uk</t>
+          <t>yuki.sakai.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1548,15 +1878,20 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>He Yuan Teng Zi</t>
+          <t>Yuan Teng Zi He</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>zcahytz@ucl.ac.uk</t>
+          <t>y.he.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
         </is>
@@ -1565,15 +1900,20 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Emilien Angles</t>
+          <t>Emilien ANGLES</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>zclmean@ucl.ac.uk</t>
+          <t>emilien.angles.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1582,15 +1922,20 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Hoi Tik Chan</t>
+          <t>hoi tik chan</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ucesh07@ucl.ac.uk</t>
+          <t>hoi.chan.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
         </is>
@@ -1599,15 +1944,20 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Ammar Hariz</t>
+          <t>Muhammad Ammar Hariz bin Mohd Shahril Izuan</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>zcemm12@ucl.ac.uk</t>
+          <t>muhammad.izuan.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1616,15 +1966,20 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Jon Fung</t>
+          <t xml:space="preserve">Jon Fung </t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>zcbt541@ucl.ac.uk</t>
+          <t>fung.lam.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1638,10 +1993,15 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>zcibdma@ucl.ac.uk</t>
+          <t>don.mathew.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1650,15 +2010,20 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Shambhavi Shambhavi Siddhida</t>
+          <t>Shambhavi Siddhida</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ucbxssi@ucl.ac.uk</t>
+          <t>Shambhavi.Siddhida.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1667,15 +2032,20 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Liu Leona</t>
+          <t>Leona Liu</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>uclqiuh@ucl.ac.uk</t>
+          <t>leona.liu.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1689,10 +2059,15 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ucahamy@ucl.ac.uk</t>
+          <t>alexander.ying.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
         <is>
           <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
@@ -1701,15 +2076,20 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Tiffany Chui</t>
+          <t xml:space="preserve">Tiffany Chui </t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>zcjtth0@ucl.ac.uk</t>
+          <t>tiffany.chui.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
         <is>
           <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1718,15 +2098,20 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Gong Yi</t>
+          <t>Yi Gong</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>zcbtyg4@ucl.ac.uk</t>
+          <t>yi.gong.26@ucl.ac.uk</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
         <is>
           <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
         </is>
@@ -1743,125 +2128,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Allocated session</t>
+          <t>UCL email address</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Huang Yalan</t>
+          <t>Yalan Huang</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zczquav@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>yalan.huang.23@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Garry Vignarajah</t>
+          <t xml:space="preserve">Garry Vignarajah </t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zcemgvi@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>garry.vignarajah.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Li Teresa</t>
+          <t>Teresa Li</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>zczqj84@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>jingtong.li.23@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tian Yihan</t>
+          <t>Yihan Tian</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>zcibyti@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>yihan.tian.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sun Tianhao</t>
+          <t>Tianhao Sun</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zchats7@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>tianhao.sun.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hyunwoo Oh</t>
+          <t>HYUNWOO Oh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>zcahhxx@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>Hyunwoo.oh.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -1873,12 +2223,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>uctysee@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>silas.eeles-nolle.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -1890,29 +2235,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>zcabnhc@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>nok.chau.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wang Bobby</t>
+          <t>Bobby Wang</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>stnzew2@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>enxun.wang.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -1924,12 +2259,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>wmhksqi@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>toto.qiao.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -1941,12 +2271,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>zctlfag@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>macaela.agyare.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -1961,26 +2286,16 @@
           <t>zcapiuv@ucl.ac.uk</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wang Yiqi</t>
+          <t>Yiqi Wang</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>zccaacc@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
         </is>
       </c>
     </row>
@@ -1992,29 +2307,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>zcftxgo@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>betty.gong.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sophia An</t>
+          <t>Yixuan An</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>zcibanb@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>sophia.an.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2026,46 +2331,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>zctp454@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>ryan.lee.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Emilien Angles</t>
+          <t>Emilien ANGLES</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>zclmean@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>emilien.angles.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tiffany Chui</t>
+          <t xml:space="preserve">Tiffany Chui </t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>zcjtth0@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>13 Oct (Tue) 6:00pm - 8:00pm @ Somers Town Community Sports Centre</t>
+          <t>tiffany.chui.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2080,23 +2370,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Allocated session</t>
+          <t>UCL email address</t>
         </is>
       </c>
     </row>
@@ -2108,29 +2393,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zcesttu@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>Tinnakrit.tuaicharoen.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vu Ngo</t>
+          <t>Ngo Hoai Vu</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zczqgox@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>hoai.ngo.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2142,29 +2417,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>stnzinq@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>yan.lin.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Wen-Han Chuang</t>
+          <t xml:space="preserve">WenHan Chuang </t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>uceswc8@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>wen-han.chuang.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2176,46 +2441,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zcahitt@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>ambuj.mittal.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Yieh, Cynthia</t>
+          <t>Cynthia Yieh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>dtnzxcy@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>xin-yu.yieh.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Allen Sun</t>
+          <t>Weilun Sun</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>zcbewsu@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>allen.sun.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2227,12 +2477,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>zchaic3@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>ian.chau.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2244,131 +2489,91 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>zccazba@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>betty.bao.23@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Angelina May</t>
+          <t xml:space="preserve">Angelina May </t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>zcemmay@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>angelina.may.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yu Sidi</t>
+          <t xml:space="preserve">Roger Song </t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ucbv968@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>haoyu.song.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ishaan Palsule</t>
+          <t>Guanchu Zong</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>zctqip0@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>guanchu.zong.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kendrix Pineda</t>
+          <t>SIDI YU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>zcecamp@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>sidi.yu.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sakai Yuki</t>
+          <t>Yuki Sakai</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>uclqysa@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>yuki.sakai.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shambhavi Shambhavi Siddhida</t>
+          <t>Shambhavi Siddhida</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ucbxssi@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>Shambhavi.Siddhida.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gong Yi</t>
+          <t>Yi Gong</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>zcbtyg4@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 1:30pm - 3:15pm @ Somers Town Community Sports Centre</t>
+          <t>yi.gong.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2383,108 +2588,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Allocated session</t>
+          <t>UCL email address</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Zhang Botao</t>
+          <t>Botao Zhang</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zcembz2@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
+          <t>botao.zhang.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Wang Sbrace</t>
+          <t>David Wang</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>stnzj39@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
+          <t>david.wang.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shen Haocong</t>
+          <t>Haocong Shen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>zcbt548@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
+          <t>haocong.shen.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Linda Cai</t>
+          <t>Liping Cai (Linda)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>qtnzlc4@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
+          <t>liping.cai.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Liu Leona</t>
+          <t>Leona Liu</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>uclqiuh@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>17 Oct (Sat) 3:15pm - 5:00pm @ Somers Town Community Sports Centre</t>
+          <t>leona.liu.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2499,57 +2674,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Allocated session</t>
+          <t>UCL email address</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tom Stevens</t>
+          <t>Thomas Stevens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zcbttj7@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>thomas.stevens.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Wu, Szu-Min</t>
+          <t>SZU MIN WU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ucenwuj@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>szu-min.wu.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2721,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ucabdp5@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>darren.prasetya.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2578,29 +2733,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ucnwiul@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>chin-chia.liu.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Skye Chang</t>
+          <t>Skye H. Y. Chang</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ucjvhc1@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>hung-yi.chang.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2612,182 +2757,127 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>yjmsjg2@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>judyta.gorska.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shi Camilla</t>
+          <t>Camilla Shi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>zctpcs8@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>camilla.shi.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Chloe Mok</t>
+          <t>Mok Ho Yi Chloe</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>zctqhym@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>chloe.chloe.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Choi Stephanie</t>
+          <t>Lok Yee Choi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>xkgtych@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>stephanie.choi.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chen Celia</t>
+          <t>Zhihan Chen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>ucbtzc0@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Song Roger</t>
+          <t>Lisa Cheok Xin Yi</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>zceehs4@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>lisa.cheok.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Zong Guanchu</t>
+          <t>Ishaan Palsule</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>zcemgzo@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>ishaan.palsule.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Lisa Cheok</t>
+          <t>Kendrix Pineda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>zcablxy@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>kendrix.pineda.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jeffrey Li</t>
+          <t>Xiaoxiao Ge</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>zctqlip@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>xiaoxiao.ge.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ammar Hariz</t>
+          <t>Muhammad Ammar Hariz bin Mohd Shahril Izuan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>zcemm12@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>muhammad.izuan.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jon Fung</t>
+          <t xml:space="preserve">Jon Fung </t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>zcbt541@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>fung.lam.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2799,12 +2889,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>zcibdma@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>don.mathew.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2816,12 +2901,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ucahamy@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 10:30am - 11:45am @ Maria Fidelis Catholic School</t>
+          <t>alexander.ying.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2836,23 +2916,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Allocated session</t>
+          <t>UCL email address</t>
         </is>
       </c>
     </row>
@@ -2864,12 +2939,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zcabvl0@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>vernados.lin.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2881,29 +2951,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zcemkc6@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>Keyi.Chen.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wen Serena</t>
+          <t>Zixun Wen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>zceizw5@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>zixun.wen.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2915,12 +2975,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>zcbtafu@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>adriel.fung.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2932,46 +2987,43 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zcftnts@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>nicole.tsoi.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rayne Zhu</t>
+          <t>Chung Lai Li Jeffrey</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>zcjthuj@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>jeffrey.li.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hoi Tik Chan</t>
+          <t>Rayne Zhu</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ucesh07@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 11:45am - 1:00pm @ Maria Fidelis Catholic School</t>
+          <t>Rayne.Zhu.26@ucl.ac.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hoi tik chan</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hoi.chan.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -2986,23 +3038,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Allocated session</t>
+          <t>UCL email address</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3061,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>uczcyha@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>Ying.han.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -3031,165 +3073,115 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zccanai@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>arjun.nair.24@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wei Haozhan</t>
+          <t>haozhan Wei</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ucbv936@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>haozhan.wei.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gordon Zhang</t>
+          <t>Boyu Zhang</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>zcembz4@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>boyu.zhang.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chou, Ying Xuan</t>
+          <t>Ying Xuan Chou</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>smgxyc0@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>ying.chou.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Zhu Mono</t>
+          <t>Mono(Yuliang) Zhu</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>zczv022@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>yuliang.zhu.25@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lih Jun Wong</t>
+          <t xml:space="preserve">Lih Jun Wong </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rmjwjwo@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>lih.wong.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Guo, Jia-Liang</t>
+          <t>Jialiang Guo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ucabuog@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>jia-liang.guo.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ellie Tsang</t>
+          <t xml:space="preserve">Ellie Tsang </t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>stnzct2@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>ellie.tsang.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jin Yunxuan</t>
+          <t>Yunxuan Jin</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>zcfayji@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>yunxuan.jin.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>He Yuan Teng Zi</t>
+          <t>Yuan Teng Zi He</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>zcahytz@ucl.ac.uk</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>18 Oct (Sun) 9:00am - 10:30am @ Maria Fidelis Catholic School (COACHED SESSION)</t>
+          <t>y.he.26@ucl.ac.uk</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3218,412 +3210,1240 @@
           <t>Email</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Full name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>UCL email address</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Sessions requested</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Austin Marsh</t>
+          <t>Chen Keyi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zcfbam0@ucl.ac.uk</t>
+          <t>zcemkc6@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Chen Keyi</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Keyi.Chen.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Superseded by a later submission</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sean Han</t>
+          <t>Yu Sidi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zctlyts@ucl.ac.uk</t>
+          <t>ucbv968@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SIDI YU</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>sidi.yu.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Superseded by a later submission</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yu Chenghao</t>
+          <t>Jiang Tracy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>zcftcy5@ucl.ac.uk</t>
+          <t>rmjwaj1@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tracy Jiang</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>rmjwaj1@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Superseded by a later submission</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ben Glover</t>
+          <t>He Yuan Teng Zi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sejkbgi@ucl.ac.uk</t>
+          <t>zcahytz@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yuan Teng Zi He</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>y.he.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 9:00am (coached); Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Superseded by a later submission</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zhang Zhuolang</t>
+          <t>Austin Marsh</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zcfthby@ucl.ac.uk</t>
+          <t>zcfbam0@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Austin Marsh</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Austin.marsh.26@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sun Yicheng</t>
+          <t>Sean Han</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>zcftys9@ucl.ac.uk</t>
+          <t>zctlyts@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sean Han</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>seanhan.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bettie Gong</t>
+          <t>Yu Chenghao</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>zcftxgo@ucl.ac.uk</t>
+          <t>zcftcy5@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Yu Chenghao</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>zcftcy5@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yu Dixiao</t>
+          <t>Ben Glover</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>zcesdy0@ucl.ac.uk</t>
+          <t>sejkbgi@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Benjamin Glover</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Benjamin.glover.26@ucl.ac.ul</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wang Jingyi</t>
+          <t>Zhang Zhuolang</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>zcemjw7@ucl.ac.uk</t>
+          <t>zcfthby@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>zhuolangzhang</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>zcfthby@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Xinyu Liu</t>
+          <t>Sun Yicheng</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>zcapiuv@ucl.ac.uk</t>
+          <t>zcftys9@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Yicheng Sun</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>zcftys9@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Sun 18 Oct 9:00am (coached); Sun 18 Oct 10:30am; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>You Qi</t>
+          <t>Bettie Gong</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ucbtqyo@ucl.ac.uk</t>
+          <t>zcftxgo@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Bettie Gong</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>bettie.gong.2026@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jen Zhang</t>
+          <t>Yu Dixiao</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>zczqz05@ucl.ac.uk</t>
+          <t>zcesdy0@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dixiao Yu</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>zcesdy0@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jon Fung</t>
+          <t>Wang Jingyi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>zcbt541@ucl.ac.uk</t>
+          <t>zcemjw7@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Jingyi Wang</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Jingyi.Wang@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Flora Zhang</t>
+          <t>Xinyu Liu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>zcjtzz5@ucl.ac.uk</t>
+          <t>zcapiuv@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>XINYU LIU</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>XINYU.LIU.25@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jiang Tracy</t>
+          <t>You Qi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>rmjwaj1@ucl.ac.uk</t>
+          <t>ucbtqyo@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Qi You</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ucbtqyo@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bosco Mak</t>
+          <t>Jen Zhang</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>zctqmw0@ucl.ac.uk</t>
+          <t>zczqz05@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Zhenyue Zhang（Jen）</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>zhenyuezhang6@gmail.com</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nonoda Keigo</t>
+          <t>Jon Fung</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>uceskn2@ucl.ac.uk</t>
+          <t>zcbt541@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Jon Fung</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>zcbt541@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm; Sun 18 Oct 10:30am; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seunghee Kwon</t>
+          <t>Flora Zhang</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>zchakwo@ucl.ac.uk</t>
+          <t>zcjtzz5@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ziyan Zhang</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ziyan.Zhang.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am; Sun 18 Oct 9:00am (coached); Sat 17 Oct 3:15pm; Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Charlotte Smith</t>
+          <t>Jiang Tracy</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>zcapcss@ucl.ac.uk</t>
+          <t>rmjwaj1@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Tracy Jiang</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>rmjwaj1@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bill Chu</t>
+          <t>Bosco Mak</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ucab398@ucl.ac.uk</t>
+          <t>zctqmw0@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Bosco Mak Wang Hei</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>bosco.mak.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sun 18 Oct 10:30am; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Putter Nutchanart</t>
+          <t>Nonoda Keigo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ucbxpnu@ucl.ac.uk</t>
+          <t>uceskn2@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Keigo Nonoda</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>keigo.nonoda.26@ucl.ac.com</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Xu Katy</t>
+          <t>Seunghee Kwon</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>dtnzugx@ucl.ac.uk</t>
+          <t>zchakwo@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Seunghee kwon</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>rachel.kwon.22@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm; Sun 18 Oct 10:30am; Sun 18 Oct 11:45am; Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ian Ng</t>
+          <t>Charlotte Smith</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>zccayhi@ucl.ac.uk</t>
+          <t>zcapcss@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Charlotte Smith</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>charlotte.smith.25@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Skyla Fan</t>
+          <t>Bill Chu</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>zcbtzf3@ucl.ac.uk</t>
+          <t>ucab398@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Bill Chu</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>jin.chu.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Queenna Huang</t>
+          <t>Putter Nutchanart</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>zcrhrbq@ucl.ac.uk</t>
+          <t>ucbxpnu@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Putter Nutchanart</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>phanthorn.nutchanart.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Vandy Wang</t>
+          <t>Xu Katy</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>uclqvxw@ucl.ac.uk</t>
+          <t>dtnzugx@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>katy xu</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>mingyi.xu.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pranav Chedella</t>
+          <t>Ian Ng</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>zctpps8@ucl.ac.uk</t>
+          <t>zccayhi@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Yan Ho Ian Ng</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>yan.ng.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lau Alexandra</t>
+          <t>Skyla Fan</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>zcfbswl@ucl.ac.uk</t>
+          <t>zcbtzf3@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Skyla Fan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>skyla.fan.24@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ethan Wang</t>
+          <t>Queenna Huang</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>zceezw7@ucl.ac.uk</t>
+          <t>zcrhrbq@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Queenna Huang</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>queenna.huang.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 3:15pm; Sun 18 Oct 10:30am</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Yuen, Constance</t>
+          <t>Vandy Wang</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>zchawty@ucl.ac.uk</t>
+          <t>uclqvxw@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Vandy Wang</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>vandy.wang.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am; Sun 18 Oct 10:30am; Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Sun 18 Oct 9:00am (coached)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Angelina Huang</t>
+          <t>Pranav Chedella</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>zcbt364@ucl.ac.uk</t>
+          <t>zctpps8@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Pranav Saketh Chedella</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pranav.chedella.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sun 18 Oct 11:45am; Sat 17 Oct 1:30pm</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pranav Suresh</t>
+          <t>Lau Alexandra</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>zcabpms@ucl.ac.uk</t>
+          <t>zcfbswl@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Alexandra Lau</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>alexandra.lau.25@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Abdullah Mohammad</t>
+          <t>Ethan Wang</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>zceeohh@ucl.ac.uk</t>
+          <t>zceezw7@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ethan wang</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>zceezw7@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm; Sun 18 Oct 10:30am; Tue 13 Oct 6:00pm</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Yuen, Constance</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>zchawty@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Yuen Wing Tung</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>wing.yuen.25@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Angelina Huang</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>zcbt364@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Angelina Huang</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>angelina.huang.25@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Pranav Suresh</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>zcabpms@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pranav mudambi suresh</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pranav.suresh.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Sun 18 Oct 9:00am (coached); Sun 18 Oct 10:30am; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Abdullah Mohammad</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>zceeohh@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Abdullah Mohammad</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>zceeohh@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Yu Zhiyuan</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>zcfbyug@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Zhiyuan Yu</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>zhiyuan.yu.26@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct 6:00pm; Sat 17 Oct 1:30pm; Sat 17 Oct 3:15pm; Sun 18 Oct 9:00am (coached); Sun 18 Oct 10:30am; Sun 18 Oct 11:45am</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Not on membership list</t>
         </is>
       </c>
     </row>

</xml_diff>